<commit_message>
new experiment setup for 80 shards
</commit_message>
<xml_diff>
--- a/files/Cases/CaseStudies_FeatureModel_Summary.xlsx
+++ b/files/Cases/CaseStudies_FeatureModel_Summary.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dilekozturk/git/esg-with-feature-expressions/files/Cases/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76C2BF79-BC9C-B949-9F7B-1627F6BF7B20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0A96C6A-01E4-B54D-A4DC-39FF1FAF174E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="580" windowWidth="25600" windowHeight="16060" xr2:uid="{95B04BAA-82AF-4E48-B751-2D8AC3B72013}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>SPL Name</t>
   </si>
@@ -66,6 +66,24 @@
   </si>
   <si>
     <t>syngo.via_VB40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hockerty Shirts Web Configurator </t>
+  </si>
+  <si>
+    <t>47 970</t>
+  </si>
+  <si>
+    <t>426 672</t>
+  </si>
+  <si>
+    <t>124 201 479 600</t>
+  </si>
+  <si>
+    <t>eMail</t>
+  </si>
+  <si>
+    <t>Soda Vending Machine</t>
   </si>
 </sst>
 </file>
@@ -124,7 +142,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -133,11 +151,21 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -472,10 +500,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{966D7892-A908-2048-9457-990E43D714FA}">
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="28.83203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.6640625" customWidth="1"/>
@@ -486,107 +514,161 @@
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" s="5"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
+      <c r="A2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B2" s="6">
+        <v>6</v>
+      </c>
+      <c r="C2" s="6">
+        <v>4</v>
+      </c>
+      <c r="D2" s="6">
+        <v>0</v>
+      </c>
+      <c r="E2" s="6">
+        <v>12</v>
+      </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" s="5"/>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
+      <c r="A3" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" s="6">
+        <v>8</v>
+      </c>
+      <c r="C3" s="6">
+        <v>5</v>
+      </c>
+      <c r="D3" s="6">
+        <v>1</v>
+      </c>
+      <c r="E3" s="6">
+        <v>23</v>
+      </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4" s="5"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
+      <c r="A4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="8">
+        <v>12</v>
+      </c>
+      <c r="C4" s="8">
+        <v>9</v>
+      </c>
+      <c r="D4" s="8">
+        <v>2</v>
+      </c>
+      <c r="E4" s="6">
+        <v>42</v>
+      </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
+      <c r="A5" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="6">
+        <v>12</v>
+      </c>
+      <c r="C5" s="6">
+        <v>9</v>
+      </c>
+      <c r="D5" s="6">
+        <v>3</v>
+      </c>
+      <c r="E5" s="6">
+        <v>498</v>
+      </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
+      <c r="A6" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="6">
+        <v>27</v>
+      </c>
+      <c r="C6" s="6">
+        <v>20</v>
+      </c>
+      <c r="D6" s="6">
+        <v>9</v>
+      </c>
+      <c r="E6" s="6">
+        <v>2664</v>
+      </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B7" s="5"/>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-      <c r="E7" s="5"/>
+      <c r="A7" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="6">
+        <v>64</v>
+      </c>
+      <c r="C7" s="6">
+        <v>48</v>
+      </c>
+      <c r="D7" s="6">
+        <v>14</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8">
-        <v>64</v>
-      </c>
-      <c r="C8">
-        <v>48</v>
-      </c>
-      <c r="D8">
-        <v>14</v>
-      </c>
-      <c r="E8" s="6">
-        <v>47.97</v>
+      <c r="A8" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="6">
+        <v>65</v>
+      </c>
+      <c r="C8" s="6">
+        <v>53</v>
+      </c>
+      <c r="D8" s="6">
+        <v>26</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="B9" s="5">
-        <v>65</v>
-      </c>
-      <c r="C9" s="5">
-        <v>53</v>
-      </c>
-      <c r="D9" s="5">
-        <v>26</v>
-      </c>
-      <c r="E9" s="5">
-        <v>426.67200000000003</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
+        <v>10</v>
+      </c>
+      <c r="B9" s="6">
+        <v>255</v>
+      </c>
+      <c r="C9" s="6">
+        <v>236</v>
+      </c>
+      <c r="D9" s="6">
+        <v>3</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15" s="1"/>
+      <c r="B15" s="1"/>
+      <c r="C15" s="1"/>
+      <c r="D15" s="1"/>
+      <c r="E15" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>